<commit_message>
Few changes date format in reports and excel export
</commit_message>
<xml_diff>
--- a/public/assets/MonthlyReportSample3test.xlsx
+++ b/public/assets/MonthlyReportSample3test.xlsx
@@ -357,7 +357,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="1" style="0" width="11.54"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="35.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -476,7 +476,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>39</v>
       </c>

</xml_diff>